<commit_message>
See update Todo list
</commit_message>
<xml_diff>
--- a/todo_list_shiny_userguide.xlsx
+++ b/todo_list_shiny_userguide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Greiner\Documents\srr_tutorial\srr_ug\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE1B365-C7EE-4F09-AED4-EDF65E3644A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B8E2189-BF96-48CF-988E-5A8F34AFB778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="20520" xr2:uid="{DA3AE3E0-2FE6-4568-A464-5696C988DC7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
     <t>Item</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>Standard layout in several parts, sigma dist, create better structure for readme distributions</t>
+  </si>
+  <si>
+    <t>Please review the update; also note the termionology for replicates instead of MoinetCarlo iterations</t>
   </si>
 </sst>
 </file>
@@ -465,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE3ABBD-2F9A-48EA-85C5-E4C1981F1E1C}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16.375" customWidth="1"/>
@@ -566,6 +569,20 @@
         <v>16</v>
       </c>
     </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>